<commit_message>
fıxed: dataset is updated
</commit_message>
<xml_diff>
--- a/ML_Diff_Report.xlsx
+++ b/ML_Diff_Report.xlsx
@@ -495,7 +495,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Oluşturulma Tarihi: 14.11.2025 22:03</t>
+          <t>Oluşturulma Tarihi: 14.11.2025 22:11</t>
         </is>
       </c>
     </row>
@@ -932,24 +932,24 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>class_0</t>
+          <t>Cultivar 1</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>class_1</t>
+          <t>Cultivar 2</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>class_2</t>
+          <t>Cultivar 3</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>class_0</t>
+          <t>Cultivar 1</t>
         </is>
       </c>
       <c r="B5" s="7" t="n">
@@ -965,7 +965,7 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>class_1</t>
+          <t>Cultivar 2</t>
         </is>
       </c>
       <c r="B6" s="8" t="n">
@@ -981,7 +981,7 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>class_2</t>
+          <t>Cultivar 3</t>
         </is>
       </c>
       <c r="B7" s="8" t="n">
@@ -1264,24 +1264,24 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>class_0</t>
+          <t>Cultivar 1</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>class_1</t>
+          <t>Cultivar 2</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>class_2</t>
+          <t>Cultivar 3</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>class_0</t>
+          <t>Cultivar 1</t>
         </is>
       </c>
       <c r="B5" s="7" t="n">
@@ -1297,7 +1297,7 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>class_1</t>
+          <t>Cultivar 2</t>
         </is>
       </c>
       <c r="B6" s="8" t="n">
@@ -1313,7 +1313,7 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>class_2</t>
+          <t>Cultivar 3</t>
         </is>
       </c>
       <c r="B7" s="8" t="n">
@@ -1596,24 +1596,24 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>class_0</t>
+          <t>Cultivar 1</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>class_1</t>
+          <t>Cultivar 2</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>class_2</t>
+          <t>Cultivar 3</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>class_0</t>
+          <t>Cultivar 1</t>
         </is>
       </c>
       <c r="B5" s="7" t="n">
@@ -1629,7 +1629,7 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>class_1</t>
+          <t>Cultivar 2</t>
         </is>
       </c>
       <c r="B6" s="8" t="n">
@@ -1645,7 +1645,7 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>class_2</t>
+          <t>Cultivar 3</t>
         </is>
       </c>
       <c r="B7" s="8" t="n">

</xml_diff>